<commit_message>
Add stg_assignments with normalised billable flag and relational tests
- latest batch, casts (date, integer), lower-cased role, Y/Yes/N/No -> boolean is_billable
- relationships test to stg_employees, accepted_values on role, not_null on the flag
- singular tests: one assignment per employee and project, one name per project code
- weekly_hours contract relaxed to a physical bound (<= 168); "> 40" is a warn-level dbt test
</commit_message>
<xml_diff>
--- a/data/project_assignments_report_invalid.xlsx
+++ b/data/project_assignments_report_invalid.xlsx
@@ -645,7 +645,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Mobile App Redesign v2</t>
+          <t>Mobile App Redesign</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Q1 Marketing Campaign</t>
+          <t>Q1 Marketing Campaign 2026</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Q1 Marketing Campaign</t>
+          <t>Q1 Marketing Campaign 2026</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">

</xml_diff>